<commit_message>
Fixes to phase two that were misssing
</commit_message>
<xml_diff>
--- a/BankCore.TestDocs/TestCases/TestDesign.xlsx
+++ b/BankCore.TestDocs/TestCases/TestDesign.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SRouge\source\repos\BankCoreSolution\BankCore.TestDocs\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F0600F2-787B-4928-82DD-C7FF51776618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8A0E4C3-75E9-4CED-97FE-8D79288E680A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Account Management" sheetId="5" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1545" uniqueCount="756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1563" uniqueCount="766">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -2383,6 +2383,37 @@
   </si>
   <si>
     <t>Rejected as expired session.</t>
+  </si>
+  <si>
+    <t>TC-INT-022</t>
+  </si>
+  <si>
+    <t>Monthly interest calculation for savings account</t>
+  </si>
+  <si>
+    <t>Account active; month-end interest run</t>
+  </si>
+  <si>
+    <t>1. Call the operation to calculate the interest</t>
+  </si>
+  <si>
+    <t>The correct interest is added to the balance of the account</t>
+  </si>
+  <si>
+    <t>TC-ACCT-021</t>
+  </si>
+  <si>
+    <t>Reject dormant to close state transfer</t>
+  </si>
+  <si>
+    <t>1.System is running
+2. Account must be dormant</t>
+  </si>
+  <si>
+    <t>1. Close the account</t>
+  </si>
+  <si>
+    <t>Account status refuses to change from dormant to closed</t>
   </si>
 </sst>
 </file>
@@ -2799,7 +2830,7 @@
     <col min="2" max="2" width="18.109375" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.33203125" style="6" customWidth="1"/>
     <col min="4" max="4" width="13.21875" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.44140625" style="6" customWidth="1"/>
     <col min="6" max="6" width="15.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.5546875" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.77734375" style="6" bestFit="1" customWidth="1"/>
@@ -3423,71 +3454,104 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="72" x14ac:dyDescent="0.3">
-      <c r="A20" s="6" t="s">
+    <row r="20" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="F20" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="J20" s="6" t="s">
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K20" s="6" t="s">
+      <c r="K20" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L20" s="6" t="s">
+      <c r="L20" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="6" t="s">
+    <row r="21" spans="1:12" ht="92.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="J21" s="6" t="s">
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="K21" s="6" t="s">
+      <c r="K21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="L21" s="6" t="s">
+      <c r="L21" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A22" s="6">
-        <f>COUNTA(A2:A21)</f>
-        <v>20</v>
+    <row r="22" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>761</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>762</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>763</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>764</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>765</v>
+      </c>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" sqref="B2:B19" xr:uid="{A905773C-25C6-4A71-9E4A-5A164C91B68D}">
       <formula1>"Account Management,Transaction Engine,Interest Calculator,Loan Processing,Reporting Engine,Authentication Module,Validation Library"</formula1>
@@ -3516,7 +3580,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A16696E0-09B8-48B2-BC8B-436903EECD32}">
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" style="6" bestFit="1" customWidth="1"/>
@@ -4453,12 +4517,6 @@
       </c>
       <c r="L29" s="6" t="s">
         <v>294</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A30" s="6">
-        <f>COUNTA($A$2:A29)</f>
-        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -4496,7 +4554,7 @@
   <cols>
     <col min="1" max="1" width="12" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.88671875" style="6" customWidth="1"/>
     <col min="4" max="4" width="13.21875" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.33203125" style="6" bestFit="1" customWidth="1"/>
@@ -5218,15 +5276,42 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A23" s="6">
-        <f>COUNTA($A$2:A22)</f>
-        <v>21</v>
+    <row r="23" spans="1:12" ht="79.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>756</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>757</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>758</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>760</v>
+      </c>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" sqref="B2:B22" xr:uid="{2B0BA792-7D4B-4585-BB42-92C2451AC05C}">
+    <dataValidation type="list" allowBlank="1" sqref="B2:B23" xr:uid="{2B0BA792-7D4B-4585-BB42-92C2451AC05C}">
       <formula1>"Account Management,Transaction Engine,Interest Calculator,Loan Processing,Reporting Engine,Authentication Module,Validation Library"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5253,7 +5338,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D5EED0C-24F1-4DBD-9942-42772A4DE538}">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" style="6" bestFit="1" customWidth="1"/>
@@ -6004,12 +6089,6 @@
       </c>
       <c r="L23" s="6" t="s">
         <v>65</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A24" s="6">
-        <f>COUNTA($A$2:A23)</f>
-        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -6041,7 +6120,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6167606B-985F-496C-BB50-FE884AE705D7}">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" style="6" bestFit="1" customWidth="1"/>
@@ -6446,12 +6525,6 @@
       </c>
       <c r="L12" s="1" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A13" s="6">
-        <f>COUNTA($A$2:A12)</f>
-        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -7079,10 +7152,6 @@
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A19" s="6">
-        <f>COUNTA($A$2:A18)</f>
-        <v>17</v>
-      </c>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
     </row>
@@ -7123,7 +7192,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6A38594-9487-456B-9157-C3DFA7AF6CBB}">
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" style="6" bestFit="1" customWidth="1"/>
@@ -7816,12 +7885,6 @@
       </c>
       <c r="L21" s="1" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A22" s="6">
-        <f>COUNTA($A$2:A21)</f>
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MSTest, NUnit, xUnit suites and coverage report
</commit_message>
<xml_diff>
--- a/BankCore.TestDocs/TestCases/TestDesign.xlsx
+++ b/BankCore.TestDocs/TestCases/TestDesign.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SRouge\source\repos\BankCoreSolution\BankCore.TestDocs\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8A0E4C3-75E9-4CED-97FE-8D79288E680A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0CE7909-A1B7-4AC8-BB42-6D631EDBD4EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Account Management" sheetId="5" r:id="rId1"/>
@@ -7503,7 +7503,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>165</v>
       </c>

</xml_diff>